<commit_message>
task-004: planilha_linhas so com comprovantes; PENDENTES p/ valor ilegivel
</commit_message>
<xml_diff>
--- a/saida/planilha/planilha_corrigida.xlsx
+++ b/saida/planilha/planilha_corrigida.xlsx
@@ -437,7 +437,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -522,7 +522,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0001_(a classificar)_04-11-2022_R$5.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0001_(a classificar)_04-11-2022_R$5.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0002_(a classificar)_04-11-2022_R$11.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0002_(a classificar)_04-11-2022_R$11.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -600,7 +600,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0003_(a classificar)_04-11-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0003_(a classificar)_04-11-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -639,7 +639,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0004_(a classificar)_04-11-2022_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0004_(a classificar)_04-11-2022_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0005_(a classificar)_21-11-2022_R$800,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0005_(a classificar)_21-11-2022_R$800,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0006_(a classificar)_28-11-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0006_(a classificar)_28-11-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -756,7 +756,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0007_(a classificar)_12-12-2022_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0007_(a classificar)_12-12-2022_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -795,7 +795,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0008_(a classificar)_14-12-2022_R$2.000,00_planifilmes_ltda.pdf</t>
+          <t>(a classificar)\0008_(a classificar)_14-12-2022_R$2.000,00_planifilmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -834,7 +834,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0009_(a classificar)_14-12-2022_R$6.000,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
+          <t>(a classificar)\0009_(a classificar)_14-12-2022_R$6.000,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -873,7 +873,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0010_(a classificar)_20-12-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0010_(a classificar)_20-12-2022_R$20.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -912,7 +912,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0011_(a classificar)_23-01-2023_R$4.500,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0011_(a classificar)_23-01-2023_R$4.500,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -951,7 +951,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0012_(a classificar)_23-01-2023_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0012_(a classificar)_23-01-2023_R$30.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -990,7 +990,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0013_(a classificar)_22-02-2023_R$19.550,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0013_(a classificar)_22-02-2023_R$19.550,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0014_(a classificar)_18-08-2023_R$380,00_radio_e_televisao_bandeirantes_s_a.pdf</t>
+          <t>(a classificar)\0014_(a classificar)_18-08-2023_R$380,00_radio_e_televisao_bandeirantes_s_a.pdf</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0015_(a classificar)_25-08-2023_R$10.500,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
+          <t>(a classificar)\0015_(a classificar)_25-08-2023_R$10.500,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0016_(a classificar)_04-09-2023_R$700,00_porviroscopio_projetos_c_c_ltda.pdf</t>
+          <t>(a classificar)\0016_(a classificar)_04-09-2023_R$700,00_porviroscopio_projetos_c_c_ltda.pdf</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0017_(a classificar)_05-09-2023_R$120,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0017_(a classificar)_05-09-2023_R$120,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0018_(a classificar)_05-09-2023_R$33.000,00_favorecido.pdf</t>
+          <t>(a classificar)\0018_(a classificar)_05-09-2023_R$33.000,00_favorecido.pdf</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0019_(a classificar)_06-09-2023_R$4.900,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
+          <t>(a classificar)\0019_(a classificar)_06-09-2023_R$4.900,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0020_(a classificar)_11-09-2023_R$3.000,00_ana_beatriz_hermanson_pomar_servicos.pdf</t>
+          <t>(a classificar)\0020_(a classificar)_11-09-2023_R$3.000,00_ana_beatriz_hermanson_pomar_servicos.pdf</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0021_(a classificar)_26-09-2023_R$11.250,00_filmes_de_taipa_prod.pdf</t>
+          <t>(a classificar)\0021_(a classificar)_26-09-2023_R$11.250,00_filmes_de_taipa_prod.pdf</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0022_(a classificar)_28-09-2023_R$15,30_casa_do_roadie.pdf</t>
+          <t>(a classificar)\0022_(a classificar)_28-09-2023_R$15,30_casa_do_roadie.pdf</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0023_(a classificar)_28-09-2023_R$350,00_casa_do_roadie.pdf</t>
+          <t>(a classificar)\0023_(a classificar)_28-09-2023_R$350,00_casa_do_roadie.pdf</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0024_(a classificar)_28-09-2023_R$8.800,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
+          <t>(a classificar)\0024_(a classificar)_28-09-2023_R$8.800,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0025_(a classificar)_29-09-2023_R$35,10_scm_prest_serv_postais_ltda.pdf</t>
+          <t>(a classificar)\0025_(a classificar)_29-09-2023_R$35,10_scm_prest_serv_postais_ltda.pdf</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0026_(a classificar)_29-09-2023_R$150,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
+          <t>(a classificar)\0026_(a classificar)_29-09-2023_R$150,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0027_(a classificar)_29-09-2023_R$500,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
+          <t>(a classificar)\0027_(a classificar)_29-09-2023_R$500,00_cityhome_servicos_imobiliarios_ltda.pdf</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0028_(a classificar)_29-09-2023_R$3.116,00_matron_informatica.pdf</t>
+          <t>(a classificar)\0028_(a classificar)_29-09-2023_R$3.116,00_matron_informatica.pdf</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0029_(a classificar)_29-09-2023_R$5.768,40_pateo_moinhos_de_vento_adm_e_part_lt.pdf</t>
+          <t>(a classificar)\0029_(a classificar)_29-09-2023_R$5.768,40_pateo_moinhos_de_vento_adm_e_part_lt.pdf</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0030_(a classificar)_29-09-2023_R$35.000,00_martina_milla_raffaelli_me.pdf</t>
+          <t>(a classificar)\0030_(a classificar)_29-09-2023_R$35.000,00_martina_milla_raffaelli_me.pdf</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0031_(a classificar)_02-10-2023_R$1.610,00_pateo_moinhos_de_vento_adm_e_part_lt.pdf</t>
+          <t>(a classificar)\0031_(a classificar)_02-10-2023_R$1.610,00_pateo_moinhos_de_vento_adm_e_part_lt.pdf</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0032_(a classificar)_03-10-2023_R$200,00_glademir_m_machado.pdf</t>
+          <t>(a classificar)\0032_(a classificar)_03-10-2023_R$200,00_glademir_m_machado.pdf</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>0033_(a classificar)_03-10-2023_R$3.020,00_matron_informatica.pdf</t>
+          <t>(a classificar)\0033_(a classificar)_03-10-2023_R$3.020,00_matron_informatica.pdf</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0034_(a classificar)_05-10-2023_R$500,00_amir_labaki.pdf</t>
+          <t>(a classificar)\0034_(a classificar)_05-10-2023_R$500,00_amir_labaki.pdf</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0035_(a classificar)_06-10-2023_R$10.500,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
+          <t>(a classificar)\0035_(a classificar)_06-10-2023_R$10.500,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0036_(a classificar)_09-10-2023_R$1.800,00_fabio_baltar_duarte.pdf</t>
+          <t>(a classificar)\0036_(a classificar)_09-10-2023_R$1.800,00_fabio_baltar_duarte.pdf</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0037_(a classificar)_09-10-2023_R$1.800,01_fabio_baltar_duarte.pdf</t>
+          <t>(a classificar)\0037_(a classificar)_09-10-2023_R$1.800,01_fabio_baltar_duarte.pdf</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0038_(a classificar)_09-10-2023_R$4.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
+          <t>(a classificar)\0038_(a classificar)_09-10-2023_R$4.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0039_(a classificar)_09-10-2023_R$7.500,00_luis_felipe_monte_cipullo_4425612981.pdf</t>
+          <t>(a classificar)\0039_(a classificar)_09-10-2023_R$7.500,00_luis_felipe_monte_cipullo_4425612981.pdf</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0040_(a classificar)_09-10-2023_R$9.502,77_mandala_tours.pdf</t>
+          <t>(a classificar)\0040_(a classificar)_09-10-2023_R$9.502,77_mandala_tours.pdf</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0041_(a classificar)_09-10-2023_R$13.500,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0041_(a classificar)_09-10-2023_R$13.500,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0042_(a classificar)_10-10-2023_R$2.300,00_faculdade_de_arquitetura_e_urbanismo.pdf</t>
+          <t>(a classificar)\0042_(a classificar)_10-10-2023_R$2.300,00_faculdade_de_arquitetura_e_urbanismo.pdf</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>0043_(a classificar)_11-10-2023_R$400,00_aamac.pdf</t>
+          <t>(a classificar)\0043_(a classificar)_11-10-2023_R$400,00_aamac.pdf</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0044_(a classificar)_11-10-2023_R$500,00_malnes_transporte_e_producao.pdf</t>
+          <t>(a classificar)\0044_(a classificar)_11-10-2023_R$500,00_malnes_transporte_e_producao.pdf</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>0045_(a classificar)_11-10-2023_R$1.000,00_idalina_s_r_silva.pdf</t>
+          <t>(a classificar)\0045_(a classificar)_11-10-2023_R$1.000,00_idalina_s_r_silva.pdf</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>0046_(a classificar)_11-10-2023_R$1.500,00_ana_beatriz_hermanson_pomar_servicos.pdf</t>
+          <t>(a classificar)\0046_(a classificar)_11-10-2023_R$1.500,00_ana_beatriz_hermanson_pomar_servicos.pdf</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0047_(a classificar)_11-10-2023_R$4.000,00_vondoc_filmes_ltda.pdf</t>
+          <t>(a classificar)\0047_(a classificar)_11-10-2023_R$4.000,00_vondoc_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>0048_(a classificar)_11-10-2023_R$9.672,00_mandala_tours.pdf</t>
+          <t>(a classificar)\0048_(a classificar)_11-10-2023_R$9.672,00_mandala_tours.pdf</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0049_(a classificar)_13-10-2023_R$300,00_ricardo_dias_santos.pdf</t>
+          <t>(a classificar)\0049_(a classificar)_13-10-2023_R$300,00_ricardo_dias_santos.pdf</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>0050_(a classificar)_13-10-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
+          <t>(a classificar)\0050_(a classificar)_13-10-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0051_(a classificar)_13-10-2023_R$2.000,00_maga_projetos_culturais.pdf</t>
+          <t>(a classificar)\0051_(a classificar)_13-10-2023_R$2.000,00_maga_projetos_culturais.pdf</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0052_(a classificar)_16-10-2023_R$1.100,00_luz_rio_locacao_de_equipamentos_cine.pdf</t>
+          <t>(a classificar)\0052_(a classificar)_16-10-2023_R$1.100,00_luz_rio_locacao_de_equipamentos_cine.pdf</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>0053_(a classificar)_17-10-2023_R$4.375,00_cristhiano_rodrigues_de_jesus_041338.pdf</t>
+          <t>(a classificar)\0053_(a classificar)_17-10-2023_R$4.375,00_cristhiano_rodrigues_de_jesus_041338.pdf</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>0054_(a classificar)_17-10-2023_R$4.900,00_claudia.pdf</t>
+          <t>(a classificar)\0054_(a classificar)_17-10-2023_R$4.900,00_claudia.pdf</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>0055_(a classificar)_18-10-2023_R$550,00_fernando_m_efron.pdf</t>
+          <t>(a classificar)\0055_(a classificar)_18-10-2023_R$550,00_fernando_m_efron.pdf</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0056_(a classificar)_24-10-2023_R$9.427,38_monica_g_p_moraes.pdf</t>
+          <t>(a classificar)\0056_(a classificar)_24-10-2023_R$9.427,38_monica_g_p_moraes.pdf</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0057_(a classificar)_25-10-2023_R$450,00_caleidoskopica_producoes.pdf</t>
+          <t>(a classificar)\0057_(a classificar)_25-10-2023_R$450,00_caleidoskopica_producoes.pdf</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0058_(a classificar)_25-10-2023_R$600,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0058_(a classificar)_25-10-2023_R$600,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>0059_(a classificar)_25-10-2023_R$816,42_sofia_v_baccarini.pdf</t>
+          <t>(a classificar)\0059_(a classificar)_25-10-2023_R$816,42_sofia_v_baccarini.pdf</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>0060_(a classificar)_25-10-2023_R$1.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
+          <t>(a classificar)\0060_(a classificar)_25-10-2023_R$1.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>0061_(a classificar)_25-10-2023_R$2.000,00_maga_projetos_culturais.pdf</t>
+          <t>(a classificar)\0061_(a classificar)_25-10-2023_R$2.000,00_maga_projetos_culturais.pdf</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>0062_(a classificar)_25-10-2023_R$3.600,00_anne_santos.pdf</t>
+          <t>(a classificar)\0062_(a classificar)_25-10-2023_R$3.600,00_anne_santos.pdf</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>0063_(a classificar)_25-10-2023_R$4.500,00_filmes_de_taipa_prod.pdf</t>
+          <t>(a classificar)\0063_(a classificar)_25-10-2023_R$4.500,00_filmes_de_taipa_prod.pdf</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>0064_(a classificar)_25-10-2023_R$4.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
+          <t>(a classificar)\0064_(a classificar)_25-10-2023_R$4.800,00_thiago_augusto_gomas_cunha_397893948.pdf</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>0065_(a classificar)_25-10-2023_R$13.500,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0065_(a classificar)_25-10-2023_R$13.500,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>0066_(a classificar)_25-10-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
+          <t>(a classificar)\0066_(a classificar)_25-10-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>0067_(a classificar)_26-10-2023_R$995,00_loc_all_de_cinema_e_televisao_limita.pdf</t>
+          <t>(a classificar)\0067_(a classificar)_26-10-2023_R$995,00_loc_all_de_cinema_e_televisao_limita.pdf</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>0068_(a classificar)_26-10-2023_R$6.550,00_grife_rio_locadora_ltda.pdf</t>
+          <t>(a classificar)\0068_(a classificar)_26-10-2023_R$6.550,00_grife_rio_locadora_ltda.pdf</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>0069_(a classificar)_26-10-2023_R$7.500,00_luis_felipe_monte_cipullo_4425612981.pdf</t>
+          <t>(a classificar)\0069_(a classificar)_26-10-2023_R$7.500,00_luis_felipe_monte_cipullo_4425612981.pdf</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>0070_(a classificar)_26-10-2023_R$11.250,00_filmes_de_taipa_prod.pdf</t>
+          <t>(a classificar)\0070_(a classificar)_26-10-2023_R$11.250,00_filmes_de_taipa_prod.pdf</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>0071_(a classificar)_30-10-2023_R$450,00_arthur_rodrigues_locacao_de_equipamento.pdf</t>
+          <t>(a classificar)\0071_(a classificar)_30-10-2023_R$450,00_arthur_rodrigues_locacao_de_equipamento.pdf</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>0072_(a classificar)_30-10-2023_R$1.500,00_martina_milla_raffaelli_me.pdf</t>
+          <t>(a classificar)\0072_(a classificar)_30-10-2023_R$1.500,00_martina_milla_raffaelli_me.pdf</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>0073_(a classificar)_30-10-2023_R$1.559,33_windsor_administracao_de_hoteis_e_se.pdf</t>
+          <t>(a classificar)\0073_(a classificar)_30-10-2023_R$1.559,33_windsor_administracao_de_hoteis_e_se.pdf</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>0074_(a classificar)_30-10-2023_R$2.529,85_windsor_administracao_de_hoteis_e_se.pdf</t>
+          <t>(a classificar)\0074_(a classificar)_30-10-2023_R$2.529,85_windsor_administracao_de_hoteis_e_se.pdf</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>0075_(a classificar)_31-10-2023_R$200,00_andre_lima_manfrim.pdf</t>
+          <t>(a classificar)\0075_(a classificar)_31-10-2023_R$200,00_andre_lima_manfrim.pdf</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>0076_(a classificar)_31-10-2023_R$320,00_jefferson_s_oliveira.pdf</t>
+          <t>(a classificar)\0076_(a classificar)_31-10-2023_R$320,00_jefferson_s_oliveira.pdf</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>0077_(a classificar)_01-11-2023_R$316,23_windsor_administracao_de_hoteis_e_se.pdf</t>
+          <t>(a classificar)\0077_(a classificar)_01-11-2023_R$316,23_windsor_administracao_de_hoteis_e_se.pdf</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>0078_(a classificar)_08-11-2023_R$4.750,00_cristhiano_rodrigues_de_jesus_041338.pdf</t>
+          <t>(a classificar)\0078_(a classificar)_08-11-2023_R$4.750,00_cristhiano_rodrigues_de_jesus_041338.pdf</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>0079_(a classificar)_14-11-2023_R$400,00_filmes_de_taipa_prod.pdf</t>
+          <t>(a classificar)\0079_(a classificar)_14-11-2023_R$400,00_filmes_de_taipa_prod.pdf</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>0080_(a classificar)_14-11-2023_R$750,00_bie_cinema_e_tv_ltda_me.pdf</t>
+          <t>(a classificar)\0080_(a classificar)_14-11-2023_R$750,00_bie_cinema_e_tv_ltda_me.pdf</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>0081_(a classificar)_14-11-2023_R$27.000,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0081_(a classificar)_14-11-2023_R$27.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>0082_(a classificar)_27-11-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
+          <t>(a classificar)\0082_(a classificar)_27-11-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>0083_(a classificar)_11-12-2023_R$2.000,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
+          <t>(a classificar)\0083_(a classificar)_11-12-2023_R$2.000,00_memoria_coletiva_imagens_e_textos_lt.pdf</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>0084_(a classificar)_20-12-2023_R$585,00_raquel_de_oliveira_lazaro_0483723061.pdf</t>
+          <t>(a classificar)\0084_(a classificar)_20-12-2023_R$585,00_raquel_de_oliveira_lazaro_0483723061.pdf</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>0085_(a classificar)_20-12-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
+          <t>(a classificar)\0085_(a classificar)_20-12-2023_R$20.625,00_fogo_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>0086_(a classificar)_24-01-2024_R$20.625,00_fogo_filmes_ltda.pdf</t>
+          <t>(a classificar)\0086_(a classificar)_24-01-2024_R$20.625,00_fogo_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>0087_(a classificar)_31-01-2024_R$487,20_in_sampa_courier_entregas_eireli.pdf</t>
+          <t>(a classificar)\0087_(a classificar)_31-01-2024_R$487,20_in_sampa_courier_entregas_eireli.pdf</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>0088_(a classificar)_23-02-2024_R$6.000,00_juba_producoes.pdf</t>
+          <t>(a classificar)\0088_(a classificar)_23-02-2024_R$6.000,00_juba_producoes.pdf</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>0089_(a classificar)_23-02-2024_R$22.500,00_fogo_filmes.pdf</t>
+          <t>(a classificar)\0089_(a classificar)_23-02-2024_R$22.500,00_fogo_filmes.pdf</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>0090_(a classificar)_07-05-2024_R$4.000,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
+          <t>(a classificar)\0090_(a classificar)_07-05-2024_R$4.000,00_julia_barbara_melo_de_sousa_40926175.pdf</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>0091_(a classificar)_31-05-2024_R$5.000,00_ganzah.pdf</t>
+          <t>(a classificar)\0091_(a classificar)_31-05-2024_R$5.000,00_ganzah.pdf</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>0092_(a classificar)_03-06-2024_R$13.500,00_fogo_filmes.pdf</t>
+          <t>(a classificar)\0092_(a classificar)_03-06-2024_R$13.500,00_fogo_filmes.pdf</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>0093_(a classificar)_03-07-2024_R$5.000,00_giovana_amano.pdf</t>
+          <t>(a classificar)\0093_(a classificar)_03-07-2024_R$5.000,00_giovana_amano.pdf</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>0094_(a classificar)_30-07-2024_R$8.000,00_brasil_imagem.pdf</t>
+          <t>(a classificar)\0094_(a classificar)_30-07-2024_R$8.000,00_brasil_imagem.pdf</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>0095_(a classificar)_09-08-2024_R$550,00_biblioteca_nacional_licenciamento.pdf</t>
+          <t>(a classificar)\0095_(a classificar)_09-08-2024_R$550,00_biblioteca_nacional_licenciamento.pdf</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>0096_(a classificar)_09-08-2024_R$2.815,00_anjo_azul_filmes_ltda.pdf</t>
+          <t>(a classificar)\0096_(a classificar)_09-08-2024_R$2.815,00_anjo_azul_filmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>0097_(a classificar)_09-08-2024_R$2.873,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
+          <t>(a classificar)\0097_(a classificar)_09-08-2024_R$2.873,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>0098_(a classificar)_09-08-2024_R$4.000,00_f_werneck_barcinski_ltda.pdf</t>
+          <t>(a classificar)\0098_(a classificar)_09-08-2024_R$4.000,00_f_werneck_barcinski_ltda.pdf</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>0099_(a classificar)_16-08-2024_R$130,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0099_(a classificar)_16-08-2024_R$130,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>0100_(a classificar)_19-08-2024_R$8.627,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
+          <t>(a classificar)\0100_(a classificar)_19-08-2024_R$8.627,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>0101_(a classificar)_03-09-2024_R$600,00_camila_braune.pdf</t>
+          <t>(a classificar)\0101_(a classificar)_03-09-2024_R$600,00_camila_braune.pdf</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -4453,7 +4453,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>0102_(a classificar)_05-09-2024_R$938,50_globo_comunicacao_e_participacoes_s_a_cnpj_27_865_757_0001_02.pdf</t>
+          <t>(a classificar)\0102_(a classificar)_05-09-2024_R$938,50_globo_comunicacao_e_participacoes_s_a_cnpj_27_865_757_0001_02.pdf</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>0103_(a classificar)_17-09-2024_R$2.250,00_lapfilme_p_c_ltda.pdf</t>
+          <t>(a classificar)\0103_(a classificar)_17-09-2024_R$2.250,00_lapfilme_p_c_ltda.pdf</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>0104_(a classificar)_17-09-2024_R$2.632,45_s_a_o_estado_de_s_paulo_cnpj_61_533_949_0001_41.pdf</t>
+          <t>(a classificar)\0104_(a classificar)_17-09-2024_R$2.632,45_s_a_o_estado_de_s_paulo_cnpj_61_533_949_0001_41.pdf</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>0105_(a classificar)_23-09-2024_R$5.500,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0105_(a classificar)_23-09-2024_R$5.500,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>0106_(a classificar)_25-09-2024_R$6.726,23_cotacao_d_t_v_m_s_a_sefic.pdf</t>
+          <t>(a classificar)\0106_(a classificar)_25-09-2024_R$6.726,23_cotacao_d_t_v_m_s_a_sefic.pdf</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>0107_(a classificar)_30-09-2024_R$700,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0107_(a classificar)_30-09-2024_R$700,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>0108_(a classificar)_30-09-2024_R$2.400,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0108_(a classificar)_30-09-2024_R$2.400,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>0109_(a classificar)_10-10-2024_R$372,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
+          <t>(a classificar)\0109_(a classificar)_10-10-2024_R$372,00_sociedade_amigos_da_cinemateca_sac.pdf</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>0110_(a classificar)_10-10-2024_R$1.836,22_cotacao_d_t_v_m_s_a_sefic.pdf</t>
+          <t>(a classificar)\0110_(a classificar)_10-10-2024_R$1.836,22_cotacao_d_t_v_m_s_a_sefic.pdf</t>
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>0111_(a classificar)_31-10-2024_R$5.000,00_porviroscopio_projetos_c_c_ltda.pdf</t>
+          <t>(a classificar)\0111_(a classificar)_31-10-2024_R$5.000,00_porviroscopio_projetos_c_c_ltda.pdf</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>0112_(a classificar)_31-10-2024_R$5.500,00_caliban_producoes_cinematograficas_l.pdf</t>
+          <t>(a classificar)\0112_(a classificar)_31-10-2024_R$5.500,00_caliban_producoes_cinematograficas_l.pdf</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>0113_(a classificar)_01-11-2024_R$140,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0113_(a classificar)_01-11-2024_R$140,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>0114_(a classificar)_04-11-2024_R$400,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0114_(a classificar)_04-11-2024_R$400,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>0115_(a classificar)_08-11-2024_R$600,00_echo_s_comunicacao_sonora_e_visual.pdf</t>
+          <t>(a classificar)\0115_(a classificar)_08-11-2024_R$600,00_echo_s_comunicacao_sonora_e_visual.pdf</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>0116_(a classificar)_08-11-2024_R$1.000,00_roberto_f_d_avila.pdf</t>
+          <t>(a classificar)\0116_(a classificar)_08-11-2024_R$1.000,00_roberto_f_d_avila.pdf</t>
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>0117_(a classificar)_12-11-2024_R$12,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0117_(a classificar)_12-11-2024_R$12,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I118" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>0118_(a classificar)_14-11-2024_R$200,00_do_contribuinte.pdf</t>
+          <t>(a classificar)\0118_(a classificar)_14-11-2024_R$200,00_do_contribuinte.pdf</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>0119_(a classificar)_28-11-2024_R$230,00_marach_servicos_audiovisuais_eireli.pdf</t>
+          <t>(a classificar)\0119_(a classificar)_28-11-2024_R$230,00_marach_servicos_audiovisuais_eireli.pdf</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>0120_(a classificar)_05-12-2024_R$1.500,00_geisa_silva_jesus.pdf</t>
+          <t>(a classificar)\0120_(a classificar)_05-12-2024_R$1.500,00_geisa_silva_jesus.pdf</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>0121_(a classificar)_05-12-2024_R$6.400,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0121_(a classificar)_05-12-2024_R$6.400,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>0122_(a classificar)_10-12-2024_R$100,00_sem_favorecido.pdf</t>
+          <t>(a classificar)\0122_(a classificar)_10-12-2024_R$100,00_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>0123_(a classificar)_17-12-2024_R$2.000,00_som_livre.pdf</t>
+          <t>(a classificar)\0123_(a classificar)_17-12-2024_R$2.000,00_som_livre.pdf</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>0124_(a classificar)_17-12-2024_R$3.000,00_editora_e_importadora_musical_fermat.pdf</t>
+          <t>(a classificar)\0124_(a classificar)_17-12-2024_R$3.000,00_editora_e_importadora_musical_fermat.pdf</t>
         </is>
       </c>
       <c r="I125" t="inlineStr"/>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>0125_(a classificar)_17-12-2024_R$3.500,00_carlos_lyra_edicoes_musicais.pdf</t>
+          <t>(a classificar)\0125_(a classificar)_17-12-2024_R$3.500,00_carlos_lyra_edicoes_musicais.pdf</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>0126_(a classificar)_17-12-2024_R$8.393,30_cotacao_d_t_v_m_s_a_sefic.pdf</t>
+          <t>(a classificar)\0126_(a classificar)_17-12-2024_R$8.393,30_cotacao_d_t_v_m_s_a_sefic.pdf</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>0127_(a classificar)_26-12-2024_R$5.000,00_giovana_amano.pdf</t>
+          <t>(a classificar)\0127_(a classificar)_26-12-2024_R$5.000,00_giovana_amano.pdf</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -5455,7 +5455,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>0128_(a classificar)_16-01-2025_R$50,00_arquivo_nacional_licenciamento.pdf</t>
+          <t>(a classificar)\0128_(a classificar)_16-01-2025_R$50,00_arquivo_nacional_licenciamento.pdf</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>0129_(a classificar)_27-02-2025_R$7.000,00_ganzah.pdf</t>
+          <t>(a classificar)\0129_(a classificar)_27-02-2025_R$7.000,00_ganzah.pdf</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>0130_(a classificar)_25-03-2025_R$626,30_sem_favorecido.pdf</t>
+          <t>(a classificar)\0130_(a classificar)_25-03-2025_R$626,30_sem_favorecido.pdf</t>
         </is>
       </c>
       <c r="I131" t="inlineStr"/>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>0131_(a classificar)_30-04-2025_R$1.200,00_planifilmes_ltda.pdf</t>
+          <t>(a classificar)\0131_(a classificar)_30-04-2025_R$1.200,00_planifilmes_ltda.pdf</t>
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>0132_(a classificar)_30-04-2025_R$3.000,00_giovana_amano.pdf</t>
+          <t>(a classificar)\0132_(a classificar)_30-04-2025_R$3.000,00_giovana_amano.pdf</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>0133_(a classificar)_07-05-2025_R$18.093,63_fogo_filmes.pdf</t>
+          <t>(a classificar)\0133_(a classificar)_07-05-2025_R$18.093,63_fogo_filmes.pdf</t>
         </is>
       </c>
       <c r="I134" t="inlineStr"/>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>0134_(a classificar)_10-11-2022_R$1.200,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0134_(a classificar)_10-11-2022_R$1.200,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -5728,7 +5728,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>0135_(a classificar)_10-11-2022_R$1.200,00_luis_felipe_labaki.pdf</t>
+          <t>(a classificar)\0135_(a classificar)_10-11-2022_R$1.200,00_luis_felipe_labaki.pdf</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>0136_(a classificar)_03-07-2023_R$25.000,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0136_(a classificar)_03-07-2023_R$25.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I137" t="inlineStr"/>
@@ -5806,7 +5806,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>0137_(a classificar)_03-07-2023_R$25.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0137_(a classificar)_03-07-2023_R$25.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I138" t="inlineStr"/>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>0138_(a classificar)_28-09-2023_R$1.000,00_sofia_v_baccarini.pdf</t>
+          <t>(a classificar)\0138_(a classificar)_28-09-2023_R$1.000,00_sofia_v_baccarini.pdf</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>0139_(a classificar)_28-09-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
+          <t>(a classificar)\0139_(a classificar)_28-09-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
         </is>
       </c>
       <c r="I140" t="inlineStr"/>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>0140_(a classificar)_29-09-2023_R$560,00_sofia_v_baccarini.pdf</t>
+          <t>(a classificar)\0140_(a classificar)_29-09-2023_R$560,00_sofia_v_baccarini.pdf</t>
         </is>
       </c>
       <c r="I141" t="inlineStr"/>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>0141_(a classificar)_29-09-2023_R$560,00_fabio_baltar_duarte.pdf</t>
+          <t>(a classificar)\0141_(a classificar)_29-09-2023_R$560,00_fabio_baltar_duarte.pdf</t>
         </is>
       </c>
       <c r="I142" t="inlineStr"/>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>0142_(a classificar)_29-09-2023_R$1.050,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0142_(a classificar)_29-09-2023_R$1.050,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I143" t="inlineStr"/>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>0143_(a classificar)_29-09-2023_R$1.050,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0143_(a classificar)_29-09-2023_R$1.050,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>0144_(a classificar)_29-09-2023_R$1.050,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0144_(a classificar)_29-09-2023_R$1.050,00_thiago_a_gomas_cunha.pdf</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -6118,7 +6118,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>0145_(a classificar)_29-09-2023_R$1.050,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0145_(a classificar)_29-09-2023_R$1.050,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>0146_(a classificar)_05-10-2023_R$700,00_edson_de_camargo_transportes.pdf</t>
+          <t>(a classificar)\0146_(a classificar)_05-10-2023_R$700,00_edson_de_camargo_transportes.pdf</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -6196,7 +6196,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>0147_(a classificar)_09-10-2023_R$240,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0147_(a classificar)_09-10-2023_R$240,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>0148_(a classificar)_09-10-2023_R$240,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0148_(a classificar)_09-10-2023_R$240,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>0149_(a classificar)_09-10-2023_R$240,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0149_(a classificar)_09-10-2023_R$240,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>0150_(a classificar)_09-10-2023_R$240,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0150_(a classificar)_09-10-2023_R$240,00_thiago_a_gomas_cunha.pdf</t>
         </is>
       </c>
       <c r="I151" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>0151_(a classificar)_13-10-2023_R$480,00_idalina_s_r_silva.pdf</t>
+          <t>(a classificar)\0151_(a classificar)_13-10-2023_R$480,00_idalina_s_r_silva.pdf</t>
         </is>
       </c>
       <c r="I152" t="inlineStr"/>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>0152_(a classificar)_13-10-2023_R$480,00_anne_c_melo_santos.pdf</t>
+          <t>(a classificar)\0152_(a classificar)_13-10-2023_R$480,00_anne_c_melo_santos.pdf</t>
         </is>
       </c>
       <c r="I153" t="inlineStr"/>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>0153_(a classificar)_13-10-2023_R$1.200,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0153_(a classificar)_13-10-2023_R$1.200,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -6469,7 +6469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>0154_(a classificar)_13-10-2023_R$1.200,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0154_(a classificar)_13-10-2023_R$1.200,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I155" t="inlineStr"/>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>0155_(a classificar)_13-10-2023_R$1.200,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0155_(a classificar)_13-10-2023_R$1.200,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I156" t="inlineStr"/>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>0156_(a classificar)_13-10-2023_R$1.200,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0156_(a classificar)_13-10-2023_R$1.200,00_thiago_a_gomas_cunha.pdf</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>0157_(a classificar)_31-10-2023_R$1.020,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0157_(a classificar)_31-10-2023_R$1.020,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>0158_(a classificar)_31-10-2023_R$1.020,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0158_(a classificar)_31-10-2023_R$1.020,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>0159_(a classificar)_31-10-2023_R$1.020,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0159_(a classificar)_31-10-2023_R$1.020,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I160" t="inlineStr"/>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>0160_(a classificar)_08-11-2023_R$300,00_bernardo_t_s_costa.pdf</t>
+          <t>(a classificar)\0160_(a classificar)_08-11-2023_R$300,00_bernardo_t_s_costa.pdf</t>
         </is>
       </c>
       <c r="I161" t="inlineStr"/>
@@ -6736,11 +6736,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>0161_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6775,11 +6771,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>0162_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6814,11 +6806,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>0163_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6853,11 +6841,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>0164_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6892,11 +6876,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>0165_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6931,11 +6911,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>0166_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -6970,11 +6946,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>0167_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -7009,11 +6981,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>0168_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
@@ -7048,11 +7016,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>0169_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
-        </is>
-      </c>
+      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: AMIR LABAKI</t>
@@ -7087,11 +7051,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>0170_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalh.pdf</t>
-        </is>
-      </c>
+      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: CAMILA LICARIAO DE CARVALHO BRAUNE 4</t>
@@ -7126,11 +7086,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>0171_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
-        </is>
-      </c>
+      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: MOG PRODUTORA</t>
@@ -7165,11 +7121,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>0172_(a classificar)_14-11-2023_R$3.724,74_monica_guimaraes_p_moraes.pdf</t>
-        </is>
-      </c>
+      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: MONICA G P MORAES</t>
@@ -7204,11 +7156,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>0173_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
-        </is>
-      </c>
+      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: BANCO RENDIMENTO S A</t>
@@ -7243,11 +7191,7 @@
           <t>AMBIGUO</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>0174_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
-        </is>
-      </c>
+      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>débito disputado por comprovantes: BANCO RENDIMENTO S A</t>
@@ -7288,7 +7232,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>0175_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0175_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -7331,7 +7275,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>0176_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0176_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -7374,7 +7318,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>0177_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0177_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -7417,7 +7361,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>0178_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0178_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -7460,7 +7404,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>0179_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0179_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -7503,7 +7447,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>0180_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0180_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -7546,7 +7490,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>0181_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0181_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -7589,7 +7533,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>0182_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0182_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -7632,7 +7576,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>0183_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
+          <t>(a classificar)\0183_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -7675,7 +7619,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>0184_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
+          <t>(a classificar)\0184_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -7718,7 +7662,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>0185_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
+          <t>(a classificar)\0185_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -7761,7 +7705,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>0186_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
+          <t>(a classificar)\0186_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -7804,7 +7748,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>0187_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0187_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -7847,7 +7791,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>0188_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0188_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -7890,7 +7834,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>0189_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
+          <t>(a classificar)\0189_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -7933,7 +7877,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>0190_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
+          <t>(a classificar)\0190_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -7976,7 +7920,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>0191_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
+          <t>(a classificar)\0191_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -8019,7 +7963,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>0192_(a classificar)_30-10-2023_R$211,50_brilho.pdf</t>
+          <t>PENDENTES\111 - 30-10-2023 - Brilho - Equipamento Luz (diária extra).pdf</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -8056,11 +8000,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>0193_(a classificar)_05-10-2023_R$700,00_edson_de_camargo.pdf</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
           <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
@@ -8095,11 +8035,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>0194_(a classificar)_10-10-2023_R$500,00_andre_lima_monfrini.pdf</t>
-        </is>
-      </c>
+      <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr">
         <is>
           <t>data/valor não bate</t>
@@ -8134,11 +8070,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>0195_(a classificar)_08-11-2023_R$300,00_bernardo_tavares_rosa.pdf</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
           <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
@@ -8173,11 +8105,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>0196_(a classificar)_26-09-2023_R$10.000,00_luis_felipe_labaki.pdf</t>
-        </is>
-      </c>
+      <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr">
         <is>
           <t>data/valor não bate</t>
@@ -8212,11 +8140,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>0197_(a classificar)_26-09-2023_R$3.000,00_ana_beatriz_hermanson_poma.pdf</t>
-        </is>
-      </c>
+      <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr">
         <is>
           <t>data/valor não bate</t>
@@ -8251,11 +8175,7 @@
           <t>SEM-COMPROVANTE</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>0198_(a classificar)_03-02-2025_R$975,04_circunstanc_1961_fsampjfn.pdf</t>
-        </is>
-      </c>
+      <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
           <t>comprovante do mesmo valor na data já vinculado a outro débito</t>

</xml_diff>

<commit_message>
task-003..006: re-baseline 95.58% (dados canônicos consistentes)
</commit_message>
<xml_diff>
--- a/saida/planilha/planilha_corrigida.xlsx
+++ b/saida/planilha/planilha_corrigida.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Pagamentos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pagamentos'!$A$1:$I$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pagamentos'!$A$1:$I$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Felipe G Rosa</t>
+          <t>Luis Felipe Labaki</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>(a classificar)\0134_(a classificar)_10-11-2022_R$1.200,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0134_(a classificar)_10-11-2022_R$1.200,00_luis_felipe_labaki.pdf</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Luis Felipe Labaki</t>
+          <t>Felipe G Rosa</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>(a classificar)\0135_(a classificar)_10-11-2022_R$1.200,00_luis_felipe_labaki.pdf</t>
+          <t>(a classificar)\0135_(a classificar)_10-11-2022_R$1.200,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Mog Produtora</t>
+          <t>Circunstancia Cinematografica e Prod</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>(a classificar)\0136_(a classificar)_03-07-2023_R$25.000,00_mog_produtora.pdf</t>
+          <t>(a classificar)\0136_(a classificar)_03-07-2023_R$25.000,00_circunstancia_cinematografica_e_prod.pdf</t>
         </is>
       </c>
       <c r="I137" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Circunstancia Cinematografica e Prod</t>
+          <t>Mog Produtora</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>(a classificar)\0137_(a classificar)_03-07-2023_R$25.000,00_circunstancia_cinematografica_e_prod.pdf</t>
+          <t>(a classificar)\0137_(a classificar)_03-07-2023_R$25.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I138" t="inlineStr"/>
@@ -5817,12 +5817,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2023-09-28</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Sofia V Baccarini</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="F139" s="2" t="n">
-        <v>1000</v>
+        <v>1524.64</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>(a classificar)\0138_(a classificar)_28-09-2023_R$1.000,00_sofia_v_baccarini.pdf</t>
+          <t>(a classificar)\0138_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -5856,12 +5856,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2023-09-28</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Andre Lima Manfrim</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -5875,7 +5875,7 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>1000</v>
+        <v>1524.64</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>(a classificar)\0139_(a classificar)_28-09-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
+          <t>(a classificar)\0139_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I140" t="inlineStr"/>
@@ -5895,12 +5895,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Sofia V Baccarini</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>560</v>
+        <v>1524.64</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>(a classificar)\0140_(a classificar)_29-09-2023_R$560,00_sofia_v_baccarini.pdf</t>
+          <t>(a classificar)\0140_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I141" t="inlineStr"/>
@@ -5934,12 +5934,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Fabio Baltar Duarte</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -5953,7 +5953,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>560</v>
+        <v>1524.64</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>(a classificar)\0141_(a classificar)_29-09-2023_R$560,00_fabio_baltar_duarte.pdf</t>
+          <t>(a classificar)\0141_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I142" t="inlineStr"/>
@@ -5973,12 +5973,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Luis F Monte Cipullo</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -5992,7 +5992,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>1050</v>
+        <v>2870.87</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>(a classificar)\0142_(a classificar)_29-09-2023_R$1.050,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0142_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I143" t="inlineStr"/>
@@ -6012,12 +6012,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Felipe G Rosa</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -6031,7 +6031,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>1050</v>
+        <v>2870.87</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>(a classificar)\0143_(a classificar)_29-09-2023_R$1.050,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0143_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -6051,12 +6051,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Thiago A Gomas Cunha</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -6070,7 +6070,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>1050</v>
+        <v>2870.87</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>(a classificar)\0144_(a classificar)_29-09-2023_R$1.050,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0144_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -6090,12 +6090,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-20</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Andre Lima Monfrini</t>
+          <t>Gol Linhas Aéreas</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>1050</v>
+        <v>2870.87</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -6118,7 +6118,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>(a classificar)\0145_(a classificar)_29-09-2023_R$1.050,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0145_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -6129,12 +6129,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2023-10-05</t>
+          <t>2023-09-28</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Edson de Camargo Transportes</t>
+          <t>Andre Lima Manfrim</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6148,7 +6148,7 @@
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>(a classificar)\0146_(a classificar)_05-10-2023_R$700,00_edson_de_camargo_transportes.pdf</t>
+          <t>(a classificar)\0146_(a classificar)_28-09-2023_R$1.000,00_andre_lima_manfrim.pdf</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -6168,12 +6168,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-09-28</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Luis F Monte Cipullo</t>
+          <t>Sofia V Baccarini</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>240</v>
+        <v>1000</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -6196,7 +6196,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>(a classificar)\0147_(a classificar)_09-10-2023_R$240,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0147_(a classificar)_28-09-2023_R$1.000,00_sofia_v_baccarini.pdf</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -6207,12 +6207,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Andre Lima Monfrini</t>
+          <t>Fabio Baltar Duarte</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -6226,7 +6226,7 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>240</v>
+        <v>560</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>(a classificar)\0148_(a classificar)_09-10-2023_R$240,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0148_(a classificar)_29-09-2023_R$560,00_fabio_baltar_duarte.pdf</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -6246,12 +6246,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Felipe G Rosa</t>
+          <t>Sofia V Baccarini</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -6265,7 +6265,7 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>240</v>
+        <v>560</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>(a classificar)\0149_(a classificar)_09-10-2023_R$240,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0149_(a classificar)_29-09-2023_R$560,00_sofia_v_baccarini.pdf</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -6285,12 +6285,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Thiago A Gomas Cunha</t>
+          <t>Luis F Monte Cipullo</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -6304,7 +6304,7 @@
         </is>
       </c>
       <c r="F151" s="2" t="n">
-        <v>240</v>
+        <v>1050</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>(a classificar)\0150_(a classificar)_09-10-2023_R$240,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0150_(a classificar)_29-09-2023_R$1.050,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I151" t="inlineStr"/>
@@ -6324,12 +6324,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Idalina S R Silva</t>
+          <t>Thiago A Gomas Cunha</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>480</v>
+        <v>1050</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>(a classificar)\0151_(a classificar)_13-10-2023_R$480,00_idalina_s_r_silva.pdf</t>
+          <t>(a classificar)\0151_(a classificar)_29-09-2023_R$1.050,00_thiago_a_gomas_cunha.pdf</t>
         </is>
       </c>
       <c r="I152" t="inlineStr"/>
@@ -6363,12 +6363,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Anne C Melo Santos</t>
+          <t>Andre Lima Monfrini</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="F153" s="2" t="n">
-        <v>480</v>
+        <v>1050</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>(a classificar)\0152_(a classificar)_13-10-2023_R$480,00_anne_c_melo_santos.pdf</t>
+          <t>(a classificar)\0152_(a classificar)_29-09-2023_R$1.050,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I153" t="inlineStr"/>
@@ -6402,12 +6402,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Andre Lima Monfrini</t>
+          <t>Felipe G Rosa</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -6421,7 +6421,7 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>1200</v>
+        <v>1050</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>(a classificar)\0153_(a classificar)_13-10-2023_R$1.200,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0153_(a classificar)_29-09-2023_R$1.050,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -6441,12 +6441,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Felipe G Rosa</t>
+          <t>Edson de Camargo Transportes</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -6460,7 +6460,7 @@
         </is>
       </c>
       <c r="F155" s="2" t="n">
-        <v>1200</v>
+        <v>700</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -6469,7 +6469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>(a classificar)\0154_(a classificar)_13-10-2023_R$1.200,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0154_(a classificar)_05-10-2023_R$700,00_edson_de_camargo_transportes.pdf</t>
         </is>
       </c>
       <c r="I155" t="inlineStr"/>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -6499,7 +6499,7 @@
         </is>
       </c>
       <c r="F156" s="2" t="n">
-        <v>1200</v>
+        <v>240</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>(a classificar)\0155_(a classificar)_13-10-2023_R$1.200,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0155_(a classificar)_09-10-2023_R$240,00_luis_f_monte_cipullo.pdf</t>
         </is>
       </c>
       <c r="I156" t="inlineStr"/>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2023-10-13</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="F157" s="2" t="n">
-        <v>1200</v>
+        <v>240</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>(a classificar)\0156_(a classificar)_13-10-2023_R$1.200,00_thiago_a_gomas_cunha.pdf</t>
+          <t>(a classificar)\0156_(a classificar)_09-10-2023_R$240,00_thiago_a_gomas_cunha.pdf</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -6558,12 +6558,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Felipe G Rosa</t>
+          <t>Andre Lima Monfrini</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -6577,7 +6577,7 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>1020</v>
+        <v>240</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>(a classificar)\0157_(a classificar)_31-10-2023_R$1.020,00_felipe_g_rosa.pdf</t>
+          <t>(a classificar)\0157_(a classificar)_09-10-2023_R$240,00_andre_lima_monfrini.pdf</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -6597,12 +6597,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Luis F Monte Cipullo</t>
+          <t>Felipe G Rosa</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -6616,7 +6616,7 @@
         </is>
       </c>
       <c r="F159" s="2" t="n">
-        <v>1020</v>
+        <v>240</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>(a classificar)\0158_(a classificar)_31-10-2023_R$1.020,00_luis_f_monte_cipullo.pdf</t>
+          <t>(a classificar)\0158_(a classificar)_09-10-2023_R$240,00_felipe_g_rosa.pdf</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
@@ -6636,12 +6636,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Andre Lima Monfrini</t>
+          <t>Amir Labaki</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>1020</v>
+        <v>945.49</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>(a classificar)\0159_(a classificar)_31-10-2023_R$1.020,00_andre_lima_monfrini.pdf</t>
+          <t>(a classificar)\0159_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
         </is>
       </c>
       <c r="I160" t="inlineStr"/>
@@ -6675,12 +6675,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2023-11-08</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Bernardo T S Costa</t>
+          <t>Anne C Melo Santos</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -6694,7 +6694,7 @@
         </is>
       </c>
       <c r="F161" s="2" t="n">
-        <v>300</v>
+        <v>480</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>(a classificar)\0160_(a classificar)_08-11-2023_R$300,00_bernardo_t_s_costa.pdf</t>
+          <t>(a classificar)\0160_(a classificar)_13-10-2023_R$480,00_anne_c_melo_santos.pdf</t>
         </is>
       </c>
       <c r="I161" t="inlineStr"/>
@@ -6714,34 +6714,38 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr"/>
+          <t>Idalina S R Silva</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>1524.64</v>
+        <v>480</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr"/>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>(a classificar)\0161_(a classificar)_13-10-2023_R$480,00_idalina_s_r_silva.pdf</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -6749,34 +6753,38 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr"/>
+          <t>Luis F Monte Cipullo</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>1524.64</v>
+        <v>1200</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr"/>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>(a classificar)\0162_(a classificar)_13-10-2023_R$1.200,00_luis_f_monte_cipullo.pdf</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -6784,34 +6792,38 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr"/>
+          <t>Thiago A Gomas Cunha</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>1524.64</v>
+        <v>1200</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>(a classificar)\0163_(a classificar)_13-10-2023_R$1.200,00_thiago_a_gomas_cunha.pdf</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -6819,34 +6831,38 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr"/>
+          <t>Andre Lima Monfrini</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>1524.64</v>
+        <v>1200</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>(a classificar)\0164_(a classificar)_13-10-2023_R$1.200,00_andre_lima_monfrini.pdf</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -6854,34 +6870,38 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr"/>
+          <t>Felipe G Rosa</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>2870.87</v>
+        <v>1200</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr"/>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>(a classificar)\0165_(a classificar)_13-10-2023_R$1.200,00_felipe_g_rosa.pdf</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -6889,34 +6909,38 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-16</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr"/>
+          <t>Camila Licariao de Carvalho Braune 4</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>36.584.511/0001-</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>2870.87</v>
+        <v>3000</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr"/>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>(a classificar)\0166_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -6924,34 +6948,38 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-25</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr"/>
+          <t>Mog Produtora</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>2870.87</v>
+        <v>10000</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>(a classificar)\0167_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -6959,34 +6987,38 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>GOL Linhas Aéreas (truncado)</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr"/>
+          <t>Luis F Monte Cipullo</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>2870.87</v>
+        <v>1020</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: GOL LINHAS AEREAS</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>(a classificar)\0168_(a classificar)_31-10-2023_R$1.020,00_luis_f_monte_cipullo.pdf</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -6994,34 +7026,38 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AMIR LABAKI (truncado)</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr"/>
+          <t>Andre Lima Monfrini</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>945.49</v>
+        <v>1020</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H170" t="inlineStr"/>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: AMIR LABAKI</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>(a classificar)\0169_(a classificar)_31-10-2023_R$1.020,00_andre_lima_monfrini.pdf</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -7029,34 +7065,38 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2023-10-16</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>CAMILA LICARIAO DE CARVALH (truncado)</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr"/>
+          <t>Felipe G Rosa</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F171" s="2" t="n">
-        <v>3000</v>
+        <v>1020</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: CAMILA LICARIAO DE CARVALHO BRAUNE 4</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>(a classificar)\0170_(a classificar)_31-10-2023_R$1.020,00_felipe_g_rosa.pdf</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -7064,34 +7104,38 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2023-10-25</t>
+          <t>2023-11-08</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>MOG PRODUTORA (truncado)</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr"/>
+          <t>Bernardo T S Costa</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>10000</v>
+        <v>300</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr"/>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: MOG PRODUTORA</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>(a classificar)\0171_(a classificar)_08-11-2023_R$300,00_bernardo_t_s_costa.pdf</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -7104,10 +7148,14 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>MONICA GUIMARAES P MORAES (truncado)</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr"/>
+          <t>Monica G P Moraes</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>(a classificar)</t>
@@ -7118,15 +7166,15 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr"/>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: MONICA G P MORAES</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>(a classificar)\0172_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -7139,10 +7187,14 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>BANCO RENDIMENTO S/A (truncado)</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr"/>
+          <t>Banco Rendimento S/a</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>(a classificar)</t>
@@ -7153,15 +7205,15 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr"/>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>débito disputado por comprovantes: BANCO RENDIMENTO S A</t>
-        </is>
-      </c>
+          <t>CONCILIADO</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>(a classificar)\0173_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -7169,32 +7221,40 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>2023-10-30</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>BANCO RENDIMENTO S/A (truncado)</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr"/>
+          <t>Brilho</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>11.400.274/0001-94</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>975.04</v>
+        <v>211.5</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr"/>
+          <t>DIVERGENTE</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>PENDENTES\111 - 30-10-2023 - Brilho - Equipamento Luz (diária extra).pdf</t>
+        </is>
+      </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>débito disputado por comprovantes: BANCO RENDIMENTO S A</t>
+          <t>data bate (2023-10-30) mas valor diverge: extrato R$211.50 vs comprovante R$0.00</t>
         </is>
       </c>
     </row>
@@ -7204,40 +7264,32 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>EDSON DE CAMARGO (truncado)</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>1524.64</v>
+        <v>700</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>(a classificar)\0175_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
         </is>
       </c>
     </row>
@@ -7247,40 +7299,32 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-10</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>Andre Lima Monfrini (truncado)</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F177" s="2" t="n">
-        <v>1524.64</v>
+        <v>500</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>(a classificar)\0176_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>data/valor não bate</t>
         </is>
       </c>
     </row>
@@ -7290,40 +7334,32 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-11-08</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>BERNARDO TAVARES ROSA (truncado)</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>1524.64</v>
+        <v>300</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>(a classificar)\0177_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
         </is>
       </c>
     </row>
@@ -7333,40 +7369,32 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-09-26</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>LUIS FELIPE LABAKI (truncado)</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>1524.64</v>
+        <v>10000</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>(a classificar)\0178_(a classificar)_20-09-2023_R$1.524,64_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>data/valor não bate</t>
         </is>
       </c>
     </row>
@@ -7376,40 +7404,32 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-09-26</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>ANA BEATRIZ HERMANSON POMA (truncado)</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F180" s="2" t="n">
-        <v>2870.87</v>
+        <v>3000</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>(a classificar)\0179_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>data/valor não bate</t>
         </is>
       </c>
     </row>
@@ -7419,40 +7439,32 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>CIRCUNSTANC 1961 FSAMPJFN (truncado)</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F181" s="2" t="n">
-        <v>2870.87</v>
+        <v>975.04</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>(a classificar)\0180_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
         </is>
       </c>
     </row>
@@ -7462,40 +7474,32 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
+          <t>BANCO RENDIMENTO S/A (truncado)</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
           <t>(a classificar)</t>
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>2870.87</v>
+        <v>975.04</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>(a classificar)\0181_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
-        </is>
-      </c>
+          <t>SEM-COMPROVANTE</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
       <c r="I182" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
         </is>
       </c>
     </row>
@@ -7505,12 +7509,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2023-09-20</t>
+          <t>2023-10-09</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Gol Linhas Aéreas</t>
+          <t>Amir Labaki</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -7524,21 +7528,21 @@
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>2870.87</v>
+        <v>945.49</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>SEM-EXTRATO</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>(a classificar)\0182_(a classificar)_20-09-2023_R$2.870,87_gol_linhas_aereas.pdf</t>
+          <t>(a classificar)\0182_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: GOL LINHAS AEREAS</t>
+          <t>sem débito correspondente</t>
         </is>
       </c>
     </row>
@@ -7548,17 +7552,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-10-16</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Amir Labaki</t>
+          <t>Camila Licariao de Carvalho Braune 4</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>11.400.274/0001-94</t>
+          <t>36.584.511/0001-</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -7567,21 +7571,21 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>945.49</v>
+        <v>3000</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>SEM-EXTRATO</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>(a classificar)\0183_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
+          <t>(a classificar)\0183_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: AMIR LABAKI</t>
+          <t>sem débito correspondente</t>
         </is>
       </c>
     </row>
@@ -7591,12 +7595,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2023-10-09</t>
+          <t>2023-10-25</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Amir Labaki</t>
+          <t>Mog Produtora</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -7610,21 +7614,21 @@
         </is>
       </c>
       <c r="F185" s="2" t="n">
-        <v>945.49</v>
+        <v>10000</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>SEM-EXTRATO</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>(a classificar)\0184_(a classificar)_09-10-2023_R$945,49_amir_labaki.pdf</t>
+          <t>(a classificar)\0184_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: AMIR LABAKI</t>
+          <t>sem débito correspondente</t>
         </is>
       </c>
     </row>
@@ -7634,17 +7638,17 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2023-10-16</t>
+          <t>2023-11-14</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Camila Licariao de Carvalho Braune 4</t>
+          <t>Monica G P Moraes</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>36.584.511/0001-</t>
+          <t>11.400.274/0001-94</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -7653,537 +7657,26 @@
         </is>
       </c>
       <c r="F186" s="2" t="n">
-        <v>3000</v>
+        <v>3724.74</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>SEM-EXTRATO</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>(a classificar)\0185_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
+          <t>(a classificar)\0185_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>comprovante disputado por débitos: CAMILA LICARIAO DE CARVALH</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="n">
-        <v>186</v>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>2023-10-16</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Camila Licariao de Carvalho Braune 4</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>36.584.511/0001-</t>
-        </is>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F187" s="2" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>(a classificar)\0186_(a classificar)_16-10-2023_R$3.000,00_camila_licariao_de_carvalho_braune_4.pdf</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: CAMILA LICARIAO DE CARVALH</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="n">
-        <v>187</v>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>2023-10-25</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Mog Produtora</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>(a classificar)\0187_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: MOG PRODUTORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>188</v>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>2023-10-25</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>Mog Produtora</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F189" s="2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>(a classificar)\0188_(a classificar)_25-10-2023_R$10.000,00_mog_produtora.pdf</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: MOG PRODUTORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="n">
-        <v>189</v>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>2023-11-14</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Monica G P Moraes</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="n">
-        <v>3724.74</v>
-      </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>(a classificar)\0189_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: MONICA GUIMARAES P MORAES</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="n">
-        <v>190</v>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>2023-11-14</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Monica G P Moraes</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F191" s="2" t="n">
-        <v>3724.74</v>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>(a classificar)\0190_(a classificar)_14-11-2023_R$3.724,74_monica_g_p_moraes.pdf</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: MONICA GUIMARAES P MORAES</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="n">
-        <v>191</v>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>2025-02-03</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>Banco Rendimento S/a</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F192" s="2" t="n">
-        <v>975.04</v>
-      </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>(a classificar)\0191_(a classificar)_03-02-2025_R$975,04_banco_rendimento_s_a.pdf</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>comprovante disputado por débitos: BANCO RENDIMENTO S A</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="n">
-        <v>192</v>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>2023-10-30</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>Brilho</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>11.400.274/0001-94</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F193" s="2" t="n">
-        <v>211.5</v>
-      </c>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>DIVERGENTE</t>
-        </is>
-      </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>PENDENTES\111 - 30-10-2023 - Brilho - Equipamento Luz (diária extra).pdf</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>data bate (2023-10-30) mas valor diverge: extrato R$211.50 vs comprovante R$0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="n">
-        <v>193</v>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>2023-10-05</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>EDSON DE CAMARGO (truncado)</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr"/>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="n">
-        <v>700</v>
-      </c>
-      <c r="G194" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H194" t="inlineStr"/>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>194</v>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>2023-10-10</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Andre Lima Monfrini (truncado)</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr"/>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F195" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr"/>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>data/valor não bate</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="n">
-        <v>195</v>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>2023-11-08</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>BERNARDO TAVARES ROSA (truncado)</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr"/>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="G196" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H196" t="inlineStr"/>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="n">
-        <v>196</v>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>2023-09-26</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>LUIS FELIPE LABAKI (truncado)</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr"/>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F197" s="2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G197" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H197" t="inlineStr"/>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>data/valor não bate</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>197</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>2023-09-26</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>ANA BEATRIZ HERMANSON POMA (truncado)</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr"/>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H198" t="inlineStr"/>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>data/valor não bate</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="n">
-        <v>198</v>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>2025-02-03</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>CIRCUNSTANC 1961 FSAMPJFN (truncado)</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>(a classificar)</t>
-        </is>
-      </c>
-      <c r="F199" s="2" t="n">
-        <v>975.04</v>
-      </c>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>SEM-COMPROVANTE</t>
-        </is>
-      </c>
-      <c r="H199" t="inlineStr"/>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>comprovante do mesmo valor na data já vinculado a outro débito</t>
+          <t>sem débito correspondente</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I199"/>
+  <autoFilter ref="A1:I186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>